<commit_message>
Updated today's matches data
</commit_message>
<xml_diff>
--- a/data/todays_matches/todays_matches.xlsx
+++ b/data/todays_matches/todays_matches.xlsx
@@ -137,8 +137,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MatchesTable" displayName="MatchesTable" ref="A1:AF4" headerRowCount="1">
-  <autoFilter ref="A1:AF4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MatchesTable" displayName="MatchesTable" ref="A1:AF9" headerRowCount="1">
+  <autoFilter ref="A1:AF9"/>
   <tableColumns count="32">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="game_week"/>
@@ -466,13 +466,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF4"/>
+  <dimension ref="A1:AF9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.2" customWidth="1" min="1" max="1"/>
     <col width="13.2" customWidth="1" min="2" max="2"/>
-    <col width="21.6" customWidth="1" min="3" max="3"/>
-    <col width="22.8" customWidth="1" min="4" max="4"/>
+    <col width="28.8" customWidth="1" min="3" max="3"/>
+    <col width="26.4" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-11-12 21:00:00</t>
+          <t>2025-11-14 00:00:00</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -676,207 +676,207 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>La Equidad</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Deportivo Pereira</t>
+          <t>Envigado</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.53</v>
+        <v>1.15</v>
       </c>
       <c r="F2" t="n">
-        <v>1.18</v>
+        <v>0.9</v>
       </c>
       <c r="G2" t="n">
-        <v>1.12</v>
+        <v>1.06</v>
       </c>
       <c r="H2" t="n">
-        <v>1.23</v>
+        <v>1.1</v>
       </c>
       <c r="I2" t="n">
-        <v>2.35</v>
+        <v>2.16</v>
       </c>
       <c r="J2" t="n">
         <v>44</v>
       </c>
       <c r="K2" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="L2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="M2" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="N2" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="O2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="P2" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="Q2" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="R2" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="S2" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="U2" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="V2" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="W2" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="X2" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="AB2" t="n">
         <v>1.9</v>
       </c>
-      <c r="R2" t="n">
-        <v>3.65</v>
-      </c>
-      <c r="S2" t="n">
-        <v>3.65</v>
-      </c>
-      <c r="T2" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="U2" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="V2" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="W2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="X2" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
       <c r="AC2" t="n">
-        <v>1.38</v>
+        <v>1.4</v>
       </c>
       <c r="AD2" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="AE2" t="n">
-        <v>2.77</v>
+        <v>2.62</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.35</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-11-12 23:30:00</t>
+          <t>2025-11-14 00:00:00</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Atlético Mineiro</t>
+          <t>Deportivo Cali</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Once Caldas</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1.13</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6</v>
+        <v>1.34</v>
       </c>
       <c r="G3" t="n">
-        <v>1.81</v>
+        <v>1.23</v>
       </c>
       <c r="H3" t="n">
-        <v>1.17</v>
+        <v>1.39</v>
       </c>
       <c r="I3" t="n">
-        <v>2.98</v>
+        <v>2.62</v>
       </c>
       <c r="J3" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="K3" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="L3" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="M3" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="N3" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="P3" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.67</v>
+        <v>1.83</v>
       </c>
       <c r="R3" t="n">
-        <v>3.23</v>
+        <v>3.08</v>
       </c>
       <c r="S3" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="T3" t="n">
-        <v>1.28</v>
+        <v>1.36</v>
       </c>
       <c r="U3" t="n">
         <v>2.15</v>
       </c>
       <c r="V3" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="W3" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="AB3" t="n">
         <v>1.93</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>2.03</v>
       </c>
       <c r="AC3" t="n">
         <v>1.4</v>
       </c>
       <c r="AD3" t="n">
-        <v>3.08</v>
+        <v>2.95</v>
       </c>
       <c r="AE3" t="n">
-        <v>2.73</v>
+        <v>2.7</v>
       </c>
       <c r="AF3" t="n">
-        <v>1.36</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-13 01:20:00</t>
+          <t>2025-11-14 00:00:00</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -884,97 +884,617 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Boyacá Chicó</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Alianza Petrolera</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.92</v>
+        <v>1.64</v>
       </c>
       <c r="F4" t="n">
-        <v>1.56</v>
+        <v>1.49</v>
       </c>
       <c r="G4" t="n">
-        <v>1.11</v>
+        <v>1.32</v>
       </c>
       <c r="H4" t="n">
-        <v>1.5</v>
+        <v>1.39</v>
       </c>
       <c r="I4" t="n">
-        <v>2.61</v>
+        <v>2.71</v>
       </c>
       <c r="J4" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="K4" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L4" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N4" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="O4" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="P4" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="Q4" t="n">
-        <v>4</v>
+        <v>1.77</v>
       </c>
       <c r="R4" t="n">
-        <v>3.36</v>
+        <v>3.2</v>
       </c>
       <c r="S4" t="n">
-        <v>1.84</v>
+        <v>4.2</v>
       </c>
       <c r="T4" t="n">
-        <v>1.35</v>
+        <v>1.27</v>
       </c>
       <c r="U4" t="n">
         <v>1.96</v>
       </c>
       <c r="V4" t="n">
-        <v>4.2</v>
+        <v>3.45</v>
       </c>
       <c r="W4" t="n">
-        <v>1.84</v>
+        <v>1.85</v>
       </c>
       <c r="X4" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-11-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Independiente Medellín</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>América de Cali</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J5" t="n">
+        <v>46</v>
+      </c>
+      <c r="K5" t="n">
+        <v>63</v>
+      </c>
+      <c r="L5" t="n">
+        <v>23</v>
+      </c>
+      <c r="M5" t="n">
+        <v>30</v>
+      </c>
+      <c r="N5" t="n">
+        <v>71</v>
+      </c>
+      <c r="O5" t="n">
+        <v>37</v>
+      </c>
+      <c r="P5" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="R5" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="S5" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="T5" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="U5" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="V5" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="X5" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="AB5" t="n">
         <v>1.88</v>
       </c>
-      <c r="Y4" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="Z4" t="n">
+      <c r="AC5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Deportivo Pasto</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Atlético Bucaramanga</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="J6" t="n">
+        <v>48</v>
+      </c>
+      <c r="K6" t="n">
+        <v>80</v>
+      </c>
+      <c r="L6" t="n">
+        <v>31</v>
+      </c>
+      <c r="M6" t="n">
+        <v>31</v>
+      </c>
+      <c r="N6" t="n">
+        <v>70</v>
+      </c>
+      <c r="O6" t="n">
+        <v>44</v>
+      </c>
+      <c r="P6" t="n">
+        <v>57</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="S6" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="T6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="U6" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="V6" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="W6" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="X6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-11-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="J7" t="n">
+        <v>55</v>
+      </c>
+      <c r="K7" t="n">
+        <v>75</v>
+      </c>
+      <c r="L7" t="n">
+        <v>33</v>
+      </c>
+      <c r="M7" t="n">
+        <v>28</v>
+      </c>
+      <c r="N7" t="n">
+        <v>72</v>
+      </c>
+      <c r="O7" t="n">
+        <v>51</v>
+      </c>
+      <c r="P7" t="n">
+        <v>49</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="R7" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="S7" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="V7" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="X7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="AA7" t="n">
         <v>1.6</v>
       </c>
-      <c r="AA4" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="AF4" t="n">
+      <c r="AB7" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Rionegro Águilas</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="J8" t="n">
+        <v>53</v>
+      </c>
+      <c r="K8" t="n">
+        <v>66</v>
+      </c>
+      <c r="L8" t="n">
+        <v>32</v>
+      </c>
+      <c r="M8" t="n">
+        <v>35</v>
+      </c>
+      <c r="N8" t="n">
+        <v>66</v>
+      </c>
+      <c r="O8" t="n">
+        <v>43</v>
+      </c>
+      <c r="P8" t="n">
+        <v>57</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="R8" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="S8" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="T8" t="n">
         <v>1.36</v>
+      </c>
+      <c r="U8" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="V8" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="W8" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="X8" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-11-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Unión Magdalena</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fortaleza CEIF</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="J9" t="n">
+        <v>48</v>
+      </c>
+      <c r="K9" t="n">
+        <v>56</v>
+      </c>
+      <c r="L9" t="n">
+        <v>26</v>
+      </c>
+      <c r="M9" t="n">
+        <v>34</v>
+      </c>
+      <c r="N9" t="n">
+        <v>67</v>
+      </c>
+      <c r="O9" t="n">
+        <v>39</v>
+      </c>
+      <c r="P9" t="n">
+        <v>61</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="R9" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="S9" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="U9" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="V9" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="W9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="X9" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>